<commit_message>
Auto update Pengadaan 2026-10-07 08:48:32
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-07).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-07).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1301651478</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1520,13 +1528,13 @@
         <v>172</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2261946920</v>
+        <v>2271451073</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -2027,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>76907682</v>
+        <v>64745634</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>17</v>
@@ -3323,7 +3331,7 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D76" s="9" t="n">
         <v>1495934570</v>
@@ -3341,7 +3349,7 @@
         <v>171985038</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J76" s="9" t="n">
         <v>1297038727</v>
@@ -3355,25 +3363,25 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3965</v>
+        <v>3938</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32750221721</v>
+        <v>32785255874</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>444</v>
+        <v>418</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6695179853</v>
+        <v>6730214006</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>444</v>
+        <v>418</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>9188540792.6</v>
+        <v>6194445968.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3521</v>
+        <v>3520</v>
       </c>
       <c r="J77" s="13" t="n">
         <v>26055041868</v>
@@ -5366,10 +5374,10 @@
         <v>23497213425.01</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>6024862460</v>
+        <v>8155480660.02</v>
       </c>
       <c r="K40" s="10" t="inlineStr">
         <is>
@@ -5576,28 +5584,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>451408750</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>273952950</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>186605952</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>186605952</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -7528,28 +7536,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>97717263058</v>
+        <v>97861227758</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64727567993</v>
+        <v>64871532693</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63141947921.41</v>
+        <v>63154109969.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>33543043877</v>
+        <v>35685824125.02</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>12</v>
@@ -8363,28 +8371,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26395646241</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24238773641</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24238773641</v>
+        <v>26395646241</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8582,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8807,34 +8815,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12005,34 +12013,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>136338797325</v>
+        <v>180774160062</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>98799023706</v>
+        <v>143234386443</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>66770344937.01</v>
+        <v>70112650313.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>62321911137</v>
+        <v>65664216513</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2915140258</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>82</v>

</xml_diff>